<commit_message>
assileye: dedup content-plan keywords (distinct long-tail per article)
Reassigned 14 articles that shared a broad head keyword to distinct long-tail
primaries (skill dedup rule) + regenerated deck + workbook. Deck re-validated:
div-balanced + nav bar renders.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/assileye/keyword-research.xlsx
+++ b/decks/assileye/keyword-research.xlsx
@@ -650,19 +650,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>How Much Does Cataract Surgery Cost in Los Angeles?</t>
+          <t>Premium Cataract Surgery in Los Angeles: Choosing the Right Advanced Lens</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>cataract surgery cost</t>
+          <t>premium cataract surgery</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2900</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>21</v>
+        <v>1000</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>71</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
@@ -692,19 +692,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Doctors Who Perform Cataract Surgery in Beverly Hills &amp; Santa Monica</t>
+          <t>Cataract Surgery in Beverly Hills: Costs, Lens Options, and What to Expect</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>doctors that do cataract surgery</t>
+          <t>cataract surgery beverly hills</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>71</v>
+        <v>110</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>10</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
@@ -734,19 +734,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Driving and Reading After Cataract Surgery: When You Can Resume</t>
+          <t>Is Cataract Surgery Safe? Risks and Safeguards Explained</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>cataract surgery recovery</t>
+          <t>is cataracts surgery safe</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>14800</v>
+        <v>6600</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
@@ -776,19 +776,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Is Cataract Surgery Painful? What Patients Actually Feel</t>
+          <t>Can Cataracts Come Back After Surgery?</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>cataract surgery</t>
+          <t>can cataracts come back</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>14800</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>40</v>
+        <v>2400</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>11</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
@@ -818,19 +818,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>How Long Does Cataract Surgery Take?</t>
+          <t>Toric IOLs: Correcting Astigmatism During Cataract Surgery</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>how long does cataract surgery take</t>
+          <t>toric iols</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>6600</v>
+        <v>1000</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
@@ -860,19 +860,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Toric IOLs: Correcting Astigmatism During Cataract Surgery</t>
+          <t>Driving and Reading After Cataract Surgery: When You Can Resume</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>toric iols</t>
+          <t>driving after cataract surgery</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1000</v>
+        <v>720</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
@@ -902,19 +902,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Life After Cataract Surgery: Your Vision, Restored</t>
+          <t>Premium IOLs Explained: Are Advanced Lenses Worth the Cost?</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>vision after cataract surgery</t>
+          <t>premium iols</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>320</v>
+        <v>260</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
@@ -944,19 +944,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Choosing Your IOL: A Patient's Guide to Lens Selection</t>
+          <t>Refractive Lens Exchange vs. LASIK: Which Fits Your Eyes?</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>iol types</t>
+          <t>refractive lens exchange vs lasik</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>170</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>20</v>
+        <v>90</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
@@ -970,7 +970,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -986,19 +986,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>When Is the Right Time for Cataract Surgery?</t>
+          <t>What Are Cataracts? Causes, Types, and Early Signs</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>cataract surgery</t>
+          <t>what are cataracts</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>14800</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>40</v>
+        <v>6600</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>31</v>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
@@ -1028,19 +1028,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>What Is an Intraocular Lens (IOL)?</t>
+          <t>The First Signs of Cataracts You Shouldn't Ignore</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>intraocular lens</t>
+          <t>signs of cataracts</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>5400</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>49</v>
+        <v>2400</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>21</v>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
@@ -1070,19 +1070,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The First Signs of Cataracts You Shouldn't Ignore</t>
+          <t>How Modern Cataract Surgery Works</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>signs of cataracts</t>
+          <t>how is cataract surgery done</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2400</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>21</v>
+        <v>1000</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>41</v>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
@@ -1112,19 +1112,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Preparing for Cataract Surgery: Your Pre-Op Checklist</t>
+          <t>When Is the Right Time for Cataract Surgery?</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>cataract eye surgery procedure</t>
+          <t>when to have cataract surgery</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>46</v>
+        <v>320</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>8</v>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
@@ -1238,19 +1238,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LASIK in Los Angeles: What Sets Our Surgeons Apart</t>
+          <t>Laser Eye Surgery Near You: Santa Monica &amp; West LA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>lasik eye surgery near me</t>
+          <t>laser eye surgery near me</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>9900</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>43</v>
+        <v>2400</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>36</v>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
@@ -1322,19 +1322,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>How Much Does LASIK Really Cost? Financing and Value</t>
+          <t>LASIK Recovery: What to Expect in the First 24 Hours</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>how much is lasik eye surgery</t>
+          <t>lasik recovery time</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>12100</v>
+        <v>3600</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
@@ -1364,19 +1364,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LASIK Success Rate: What the Numbers Show</t>
+          <t>Is LASIK Worth It? Weighing the Long-Term Value</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>lasik success rate</t>
+          <t>is lasik worth it</t>
         </is>
       </c>
       <c r="E20" t="n">
         <v>2400</v>
       </c>
-      <c r="F20" s="2" t="n">
-        <v>21</v>
+      <c r="F20" s="5" t="n">
+        <v>9</v>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
@@ -1908,19 +1908,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Pterygium Removal: Treating 'Surfer's Eye'</t>
+          <t>Corneal Cross-Linking for Keratoconus: How It Halts Progression</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>pterygium surfer's eye</t>
+          <t>corneal cross linking</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>14800</v>
+        <v>4400</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
@@ -1950,19 +1950,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Eye Freckle (Conjunctival Nevus) Removal: What to Expect</t>
+          <t>Treating Eye Floaters: When to Worry and What Helps</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>eye freckle removal</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>170</v>
-      </c>
+          <t>eye floaters treatment</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" s="5" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
@@ -2034,19 +2032,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Meibomian Gland Dysfunction: A Hidden Cause of Dry Eye</t>
+          <t>What Your Eye Exam Really Checks For</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>meibomian gland</t>
+          <t>eye exam</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>14800</v>
-      </c>
-      <c r="F36" s="2" t="n">
-        <v>30</v>
+        <v>12100</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>43</v>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
@@ -2076,19 +2074,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Why Do I Have Small Pupils? Causes and When to Worry</t>
+          <t>Foods and Vitamins for Healthy Eyes</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>small pupils</t>
+          <t>foods for eye health</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>5400</v>
+        <v>2400</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
@@ -2118,19 +2116,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Types of Color Blindness, Explained</t>
+          <t>Diabetic Eye Disease: Protecting Vision With Diabetes</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>types of color blindness</t>
+          <t>diabetic</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>390</v>
-      </c>
-      <c r="F38" s="2" t="n">
-        <v>32</v>
+        <v>320</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>7</v>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
@@ -2160,19 +2158,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Common Eye Conditions and Their Warning Signs</t>
+          <t>What Is Keratoconus? Causes, Symptoms, and Treatment</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>common eye conditions</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>170</v>
-      </c>
-      <c r="F39" s="2" t="n">
-        <v>23</v>
+          <t>what is keratoconus</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
@@ -2207,7 +2203,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>blepharoplasty</t>
+          <t>blepharoplasty recovery</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -2328,12 +2324,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Premium Cataract Surgery in Los Angeles: Choosing the Right Advanced Lens</t>
+          <t>Choosing the Best Cataract Surgeon in Los Angeles: What to Look For</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>premium cataract surgery</t>
+          <t>cataract surgeon</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -2412,19 +2408,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Cataract Surgery Restrictions: What to Avoid While Healing</t>
+          <t>Cataract Surgery Options: Standard vs. Laser-Assisted</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>cataract surgery recovery</t>
+          <t>cataracts surgery options</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>14800</v>
+        <v>6600</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
@@ -2438,7 +2434,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J45" t="inlineStr"/>
@@ -2454,19 +2450,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Is Cataract Surgery Safe? Risks and Safeguards Explained</t>
+          <t>PanOptix vs. TECNIS: Comparing Premium Trifocal Lenses</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>is cataracts surgery safe</t>
+          <t>panoptix vs tecnis</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>6600</v>
-      </c>
-      <c r="F46" s="4" t="n">
-        <v>60</v>
+        <v>1900</v>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>8</v>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
@@ -2480,7 +2476,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J46" t="inlineStr"/>
@@ -2496,19 +2492,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Refractive Lens Exchange vs. LASIK: Which Fits Your Eyes?</t>
+          <t>What Happens During Cataract Surgery: A Step-by-Step Guide</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>refractive lens exchange</t>
+          <t>how does cataract surgery work</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>6600</v>
-      </c>
-      <c r="F47" s="2" t="n">
-        <v>22</v>
+        <v>1000</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>71</v>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
@@ -2522,7 +2518,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Consider</t>
         </is>
       </c>
       <c r="J47" t="inlineStr"/>
@@ -2538,19 +2534,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>What Happens During Cataract Surgery: A Step-by-Step Guide</t>
+          <t>Multifocal vs. Monofocal IOLs: Which Lens Is Right for You?</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>how does cataract surgery work</t>
+          <t>multifocal iols</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F48" s="4" t="n">
-        <v>71</v>
+        <v>390</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>18</v>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
@@ -2564,7 +2560,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J48" t="inlineStr"/>
@@ -2580,19 +2576,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Premium IOLs Explained: Are Advanced Lenses Worth the Cost?</t>
+          <t>Choosing Your IOL: A Patient's Guide to Lens Selection</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>premium iols</t>
+          <t>iol types</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>260</v>
-      </c>
-      <c r="F49" s="5" t="n">
-        <v>9</v>
+        <v>170</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>20</v>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
@@ -2622,17 +2618,15 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Is Refractive Lens Exchange Safe? Benefits and Risks</t>
+          <t>EDOF Lenses: Extended Depth of Focus for Everyday Vision</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>refractive lens exchange risks</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>140</v>
-      </c>
+          <t>edof lenses</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
       <c r="F50" s="5" t="n">
         <v>0</v>
       </c>
@@ -2664,19 +2658,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Posterior Capsule Opacification: The 'Secondary Cataract'</t>
+          <t>What Is an Intraocular Lens (IOL)?</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>cataract surgery</t>
+          <t>intraocular lens</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>14800</v>
+        <v>5400</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
@@ -2706,19 +2700,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>How Cataracts Change Your Vision Over Time</t>
+          <t>Types of Cataracts: Nuclear, Cortical, and Beyond</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>cataract vision</t>
+          <t>types of cataracts</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>3600</v>
-      </c>
-      <c r="F52" s="2" t="n">
-        <v>27</v>
+        <v>2400</v>
+      </c>
+      <c r="F52" s="5" t="n">
+        <v>14</v>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
@@ -2748,19 +2742,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Types of Cataracts: Nuclear, Cortical, and Beyond</t>
+          <t>Preparing for Cataract Surgery: Your Pre-Op Checklist</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>types of cataracts</t>
+          <t>cataract eye surgery procedure</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>2400</v>
-      </c>
-      <c r="F53" s="5" t="n">
-        <v>14</v>
+        <v>1000</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>46</v>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
@@ -2790,19 +2784,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Cataracts vs. Glaucoma: Two Conditions, Explained</t>
+          <t>What Is Refractive Lens Exchange (RLE)?</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>what are the symptoms of cataracts and glaucoma</t>
+          <t>what is rle</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>480</v>
-      </c>
-      <c r="F54" s="2" t="n">
-        <v>21</v>
+        <v>210</v>
+      </c>
+      <c r="F54" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
@@ -2832,12 +2826,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>What Causes Cataracts? Risk Factors Explained</t>
+          <t>Cataracts and Diabetes: What Patients Should Know</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>cataract eyes</t>
+          <t>cataracts and diabetes</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2872,19 +2866,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>LASIK in Beverly Hills: Candidacy, Cost, and Consultation</t>
+          <t>LASIK Eye Surgery Near You: Choosing a Los Angeles Surgeon</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>lasik</t>
+          <t>lasik near me</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>27100</v>
-      </c>
-      <c r="F56" s="2" t="n">
-        <v>28</v>
+        <v>12100</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>46</v>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
@@ -2914,19 +2908,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Laser Eye Surgery Near You: Santa Monica &amp; West LA</t>
+          <t>EVO ICL in Los Angeles: The Implantable Lens Alternative to LASIK</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>laser eye surgery near me</t>
+          <t>implantable contact lens</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>2400</v>
+        <v>1300</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
@@ -2998,19 +2992,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LASIK Recovery: What to Expect in the First 24 Hours</t>
+          <t>LASIK for Astigmatism: Can Laser Surgery Correct It?</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>lasik recovery time</t>
+          <t>astigmatism laser eye surgery</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>3600</v>
-      </c>
-      <c r="F59" s="2" t="n">
-        <v>23</v>
+        <v>2900</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>42</v>
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
@@ -3586,19 +3580,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Dry Eye Relief: From Drops to Advanced Treatments</t>
+          <t>Eye Freckle (Conjunctival Nevus) Removal: What to Expect</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>dry eye</t>
+          <t>eye freckle removal</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>8100</v>
-      </c>
-      <c r="F73" s="4" t="n">
-        <v>40</v>
+        <v>170</v>
+      </c>
+      <c r="F73" s="5" t="n">
+        <v>13</v>
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
@@ -3670,19 +3664,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Eye Floaters and Flashes: When to See a Specialist</t>
+          <t>How to Get Rid of a Stye: Causes and Treatment</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>floaters</t>
+          <t>stye in the eye</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>22200</v>
+        <v>14800</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
@@ -3712,19 +3706,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>What Your Eye Exam Really Checks For</t>
+          <t>Stye vs. Chalazion: How to Tell the Difference</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>eye exam</t>
+          <t>stye vs chalazion</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>12100</v>
-      </c>
-      <c r="F76" s="4" t="n">
-        <v>43</v>
+        <v>6600</v>
+      </c>
+      <c r="F76" s="5" t="n">
+        <v>17</v>
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
@@ -3754,19 +3748,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>What Is Keratoconus? Causes, Symptoms, and Treatment</t>
+          <t>Eye Floaters and Flashes: When to See a Specialist</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>keratoconus</t>
+          <t>eye floaters and flashes</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>4400</v>
+        <v>1300</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="G77" s="8" t="inlineStr">
         <is>
@@ -3796,19 +3790,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Diabetic Eye Disease: Protecting Vision With Diabetes</t>
+          <t>Poor Vision: Common Causes and Correction Options</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>diabetic</t>
+          <t>what is considered poor vision</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>320</v>
-      </c>
-      <c r="F78" s="5" t="n">
-        <v>7</v>
+        <v>210</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>28</v>
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
@@ -3885,7 +3879,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>blepharoplasty</t>
+          <t>blepharoplasty candidate</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -3922,19 +3916,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>When Drooping Eyelids Affect Your Sight</t>
+          <t>Droopy Eyelids: Medical and Cosmetic Solutions</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>eyelid surgery</t>
+          <t>droopy eyelid</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>3600</v>
-      </c>
-      <c r="F81" s="5" t="n">
-        <v>14</v>
+        <v>2400</v>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>36</v>
       </c>
       <c r="G81" s="9" t="inlineStr">
         <is>
@@ -3964,7 +3958,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Cataract Surgery in Beverly Hills: Costs, Lens Options, and What to Expect</t>
+          <t>How Much Does Cataract Surgery Cost in Los Angeles?</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4006,12 +4000,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Choosing the Best Cataract Surgeon in Los Angeles: What to Look For</t>
+          <t>Doctors Who Perform Cataract Surgery in Beverly Hills &amp; Santa Monica</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>cataract surgeon</t>
+          <t>doctors that do cataract surgery</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -4090,19 +4084,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Can Cataracts Come Back After Surgery?</t>
+          <t>How Long Does Cataract Surgery Take?</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>cataract surgery</t>
+          <t>how long does cataract surgery take</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>14800</v>
-      </c>
-      <c r="F85" s="4" t="n">
-        <v>40</v>
+        <v>6600</v>
+      </c>
+      <c r="F85" s="5" t="n">
+        <v>8</v>
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
@@ -4132,19 +4126,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Cataract Surgery Options: Standard vs. Laser-Assisted</t>
+          <t>Is Cataract Surgery Painful? What Patients Actually Feel</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>cataracts surgery options</t>
+          <t>is cataract surgery painful</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>6600</v>
-      </c>
-      <c r="F86" s="4" t="n">
-        <v>60</v>
+        <v>1900</v>
+      </c>
+      <c r="F86" s="5" t="n">
+        <v>2</v>
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
@@ -4158,7 +4152,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Consider</t>
         </is>
       </c>
       <c r="J86" t="inlineStr"/>
@@ -4174,19 +4168,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>PanOptix vs. TECNIS: Comparing Premium Trifocal Lenses</t>
+          <t>Cataract Surgery Restrictions: What to Avoid While Healing</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>toric iols</t>
+          <t>cataract surgery restrictions</t>
         </is>
       </c>
       <c r="E87" t="n">
         <v>1000</v>
       </c>
-      <c r="F87" s="5" t="n">
-        <v>18</v>
+      <c r="F87" s="4" t="n">
+        <v>71</v>
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
@@ -4200,7 +4194,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Consider</t>
         </is>
       </c>
       <c r="J87" t="inlineStr"/>
@@ -4216,19 +4210,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Multifocal vs. Monofocal IOLs: Which Lens Is Right for You?</t>
+          <t>Life After Cataract Surgery: Your Vision, Restored</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>multifocal iols</t>
+          <t>vision after cataract surgery</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>390</v>
+        <v>320</v>
       </c>
       <c r="F88" s="5" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
@@ -4242,7 +4236,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Consider</t>
         </is>
       </c>
       <c r="J88" t="inlineStr"/>
@@ -4258,19 +4252,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>EDOF Lenses: Extended Depth of Focus for Everyday Vision</t>
+          <t>Is Refractive Lens Exchange Safe? Benefits and Risks</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>premium iols</t>
+          <t>refractive lens exchange risks</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>260</v>
+        <v>140</v>
       </c>
       <c r="F89" s="5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
@@ -4300,19 +4294,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>The Disadvantages of Cataract Surgery: An Honest Look</t>
+          <t>What Causes Cataracts? Risk Factors Explained</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>cataract surgery</t>
+          <t>what causes cataracts</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>14800</v>
-      </c>
-      <c r="F90" s="4" t="n">
-        <v>40</v>
+        <v>9900</v>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>20</v>
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
@@ -4342,19 +4336,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>What Are Cataracts? Causes, Types, and Early Signs</t>
+          <t>How Cataracts Change Your Vision Over Time</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>what are cataracts</t>
+          <t>cataract vision</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>6600</v>
+        <v>3600</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
@@ -4389,14 +4383,14 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>astigmatism laser eye surgery</t>
+          <t>cataract surgery astigmatism</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>2900</v>
+        <v>1000</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
@@ -4426,19 +4420,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>How Modern Cataract Surgery Works</t>
+          <t>Cataracts vs. Glaucoma: Two Conditions, Explained</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>how is cataract surgery done</t>
+          <t>what are the symptoms of cataracts and glaucoma</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F93" s="4" t="n">
-        <v>41</v>
+        <v>480</v>
+      </c>
+      <c r="F93" s="2" t="n">
+        <v>21</v>
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
@@ -4468,19 +4462,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>What Is Refractive Lens Exchange (RLE)?</t>
+          <t>The Disadvantages of Cataract Surgery: An Honest Look</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>what is rle</t>
+          <t>disadvantages of cataract surgery</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>210</v>
+        <v>70</v>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
@@ -4510,12 +4504,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Cataracts and Diabetes: What Patients Should Know</t>
+          <t>Posterior Capsule Opacification: The 'Secondary Cataract'</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>cataract eyes</t>
+          <t>posterior capsule opacification</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -4550,19 +4544,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>LASIK Eye Surgery Near You: Choosing a Los Angeles Surgeon</t>
+          <t>LASIK in Los Angeles: What Sets Our Surgeons Apart</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>lasik near me</t>
+          <t>lasik eye surgery near me</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>12100</v>
+        <v>9900</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G96" s="6" t="inlineStr">
         <is>
@@ -4592,19 +4586,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>EVO ICL in Los Angeles: The Implantable Lens Alternative to LASIK</t>
+          <t>LASIK in Beverly Hills: Candidacy, Cost, and Consultation</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>implantable contact lens</t>
+          <t>lasik beverly hills</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>1300</v>
+        <v>390</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
@@ -4634,19 +4628,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Is LASIK Worth It? Weighing the Long-Term Value</t>
+          <t>How Much Does LASIK Really Cost? Financing and Value</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>lasik</t>
+          <t>how much is lasik eye surgery</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>27100</v>
+        <v>12100</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G98" s="6" t="inlineStr">
         <is>
@@ -4676,19 +4670,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>LASIK for Astigmatism: Can Laser Surgery Correct It?</t>
+          <t>LASIK Success Rate: What the Numbers Show</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>astigmatism laser eye surgery</t>
+          <t>lasik success rate</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>2900</v>
-      </c>
-      <c r="F99" s="4" t="n">
-        <v>42</v>
+        <v>2400</v>
+      </c>
+      <c r="F99" s="2" t="n">
+        <v>21</v>
       </c>
       <c r="G99" s="6" t="inlineStr">
         <is>
@@ -5222,19 +5216,19 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Treating Eye Floaters: When to Worry and What Helps</t>
+          <t>Pterygium Removal: Treating 'Surfer's Eye'</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>floaters</t>
+          <t>pterygium surfer's eye</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>22200</v>
-      </c>
-      <c r="F112" s="4" t="n">
-        <v>51</v>
+        <v>14800</v>
+      </c>
+      <c r="F112" s="2" t="n">
+        <v>28</v>
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
@@ -5264,19 +5258,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Corneal Cross-Linking for Keratoconus: How It Halts Progression</t>
+          <t>Dry Eye Relief: From Drops to Advanced Treatments</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>keratoconus</t>
-        </is>
-      </c>
-      <c r="E113" t="n">
-        <v>4400</v>
-      </c>
-      <c r="F113" s="2" t="n">
-        <v>28</v>
+          <t>dry eye relief</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
@@ -5348,19 +5340,19 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>How to Get Rid of a Stye: Causes and Treatment</t>
+          <t>Meibomian Gland Dysfunction: A Hidden Cause of Dry Eye</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>stye in the eye</t>
+          <t>meibomian gland</t>
         </is>
       </c>
       <c r="E115" t="n">
         <v>14800</v>
       </c>
-      <c r="F115" s="4" t="n">
-        <v>41</v>
+      <c r="F115" s="2" t="n">
+        <v>30</v>
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
@@ -5390,19 +5382,19 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Stye vs. Chalazion: How to Tell the Difference</t>
+          <t>Why Do I Have Small Pupils? Causes and When to Worry</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>stye vs chalazion</t>
+          <t>small pupils</t>
         </is>
       </c>
       <c r="E116" t="n">
-        <v>6600</v>
-      </c>
-      <c r="F116" s="5" t="n">
-        <v>17</v>
+        <v>5400</v>
+      </c>
+      <c r="F116" s="2" t="n">
+        <v>37</v>
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
@@ -5432,19 +5424,19 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Foods and Vitamins for Healthy Eyes</t>
+          <t>Types of Color Blindness, Explained</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>foods for eye health</t>
+          <t>types of color blindness</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>2400</v>
+        <v>390</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
@@ -5474,19 +5466,19 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Poor Vision: Common Causes and Correction Options</t>
+          <t>Common Eye Conditions and Their Warning Signs</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>what is considered poor vision</t>
+          <t>common eye conditions</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="F118" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
@@ -5563,14 +5555,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>eyelid surgery</t>
-        </is>
-      </c>
-      <c r="E120" t="n">
-        <v>3600</v>
-      </c>
+          <t>functional vs cosmetic eyelid surgery</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
       <c r="F120" s="5" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G120" s="9" t="inlineStr">
         <is>
@@ -5600,12 +5590,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Droopy Eyelids: Medical and Cosmetic Solutions</t>
+          <t>When Drooping Eyelids Affect Your Sight</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>droopy eyelid</t>
+          <t>droopy eyelid surgery</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -6510,9 +6500,9 @@
           <t>Sub page</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -9051,9 +9041,9 @@
           <t>Sub page</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G103" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -9348,9 +9338,9 @@
           <t>Sub page</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G112" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -10305,9 +10295,9 @@
           <t>Sub page</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G141" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -17004,9 +16994,9 @@
           <t>Sub page</t>
         </is>
       </c>
-      <c r="G344" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G344" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -60729,9 +60719,9 @@
           <t>Pillar page</t>
         </is>
       </c>
-      <c r="G1669" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G1669" s="11" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -89905,14 +89895,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>is cataract surgery painful</t>
+          <t>pain in inner corner of eye</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1900</v>
+        <v>1300</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
@@ -89928,37 +89918,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pain in inner corner of eye</t>
+          <t>permanent contact lenses</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>1300</v>
       </c>
       <c r="C5" t="n">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Emergency/medical — liability</t>
+          <t>Optical retail — wrong intent</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Acute-symptom queries carry medical-claim liability and are owned by Mayo/WebMD; covered only where they route to a relevant specialty.</t>
+          <t>Shopping intent for glasses/contacts; owned by retailers (Warby Parker, 1-800 Contacts), not a surgical practice.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>permanent contact lenses</t>
+          <t>implantable contact lenses</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>1300</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
@@ -89974,37 +89964,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>implantable contact lenses</t>
+          <t>sudden vision changes</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1300</v>
+        <v>1000</v>
       </c>
       <c r="C7" t="n">
         <v>26</v>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Optical retail — wrong intent</t>
+          <t>Emergency/medical — liability</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Shopping intent for glasses/contacts; owned by retailers (Warby Parker, 1-800 Contacts), not a surgical practice.</t>
+          <t>Acute-symptom queries carry medical-claim liability and are owned by Mayo/WebMD; covered only where they route to a relevant specialty.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>sudden vision changes</t>
+          <t>sudden bloodshot eye</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>1000</v>
       </c>
       <c r="C8" t="n">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
@@ -90020,14 +90010,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>sudden bloodshot eye</t>
+          <t>does glaucoma cause blindness</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>1000</v>
       </c>
       <c r="C9" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
@@ -90043,37 +90033,37 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>does glaucoma cause blindness</t>
+          <t>glaucoma symptoms</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1000</v>
+        <v>60500</v>
       </c>
       <c r="C10" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Emergency/medical — liability</t>
+          <t>Lower priority / future months</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Acute-symptom queries carry medical-claim liability and are owned by Mayo/WebMD; covered only where they route to a relevant specialty.</t>
+          <t>Solid keyword but below the cataract-first cut line for the first 90 days; queued as overflow in the Universe tab.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>glaucoma symptoms</t>
+          <t>vision laser treatment</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>60500</v>
+        <v>33100</v>
       </c>
       <c r="C11" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
@@ -90089,14 +90079,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>vision laser treatment</t>
+          <t>eye test</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>33100</v>
+        <v>22200</v>
       </c>
       <c r="C12" t="n">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
@@ -90112,14 +90102,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>eye test</t>
+          <t>cataract symptoms</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>22200</v>
       </c>
       <c r="C13" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
@@ -90135,14 +90125,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cataract symptoms</t>
+          <t>sign and symptoms of cataracts</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>22200</v>
+        <v>18100</v>
       </c>
       <c r="C14" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
@@ -90158,14 +90148,14 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sign and symptoms of cataracts</t>
+          <t>how much does lasik cost</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18100</v>
+        <v>14800</v>
       </c>
       <c r="C15" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
@@ -90181,14 +90171,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>how much does lasik cost</t>
+          <t>eye examination glaucoma</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>14800</v>
+        <v>12100</v>
       </c>
       <c r="C16" t="n">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
@@ -90204,14 +90194,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>eye examination glaucoma</t>
+          <t>glaucoma surgery</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>12100</v>
       </c>
       <c r="C17" t="n">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
@@ -90227,14 +90217,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>glaucoma surgery</t>
+          <t>cataract after operation</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>12100</v>
       </c>
       <c r="C18" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
@@ -90250,14 +90240,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cataract after operation</t>
+          <t>how much is lasik</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>12100</v>
       </c>
       <c r="C19" t="n">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
@@ -90273,14 +90263,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>how much is lasik</t>
+          <t>cost laser eye</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>12100</v>
       </c>
       <c r="C20" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
@@ -90296,14 +90286,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cost laser eye</t>
+          <t>eye laser vision correction</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>12100</v>
       </c>
       <c r="C21" t="n">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
@@ -90319,14 +90309,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>eye laser vision correction</t>
+          <t>eye diseases</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>12100</v>
       </c>
       <c r="C22" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
@@ -90342,14 +90332,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>eye diseases</t>
+          <t>eye pressure</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>12100</v>
+        <v>9900</v>
       </c>
       <c r="C23" t="n">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
@@ -90365,14 +90355,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>eye pressure</t>
+          <t>charges for eye test</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>9900</v>
       </c>
       <c r="C24" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
@@ -90388,14 +90378,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>charges for eye test</t>
+          <t>eye exam cost</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>9900</v>
       </c>
       <c r="C25" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
@@ -90411,7 +90401,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>eye exam cost</t>
+          <t>cataract procedure recovery</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -90434,14 +90424,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>cataract procedure recovery</t>
+          <t>lasik eye surgery price</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>9900</v>
       </c>
       <c r="C27" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
@@ -90457,14 +90447,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>lasik eye surgery price</t>
+          <t>surgery cost lasik</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>9900</v>
       </c>
       <c r="C28" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
@@ -90480,14 +90470,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>surgery cost lasik</t>
+          <t>discount eye tests</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>9900</v>
+        <v>8100</v>
       </c>
       <c r="C29" t="n">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
@@ -90503,14 +90493,14 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>what causes cataracts</t>
+          <t>laser eye surgery cost</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>9900</v>
+        <v>8100</v>
       </c>
       <c r="C30" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
@@ -90526,14 +90516,14 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>discount eye tests</t>
+          <t>eye problems</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>8100</v>
       </c>
       <c r="C31" t="n">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
@@ -90549,14 +90539,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>laser eye surgery cost</t>
+          <t>eye test fees</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>8100</v>
+        <v>6600</v>
       </c>
       <c r="C32" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
@@ -90572,14 +90562,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>eye problems</t>
+          <t>comprehensive eye exam</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>8100</v>
+        <v>6600</v>
       </c>
       <c r="C33" t="n">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
@@ -90595,14 +90585,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>eye test fees</t>
+          <t>cost of cataract surgery</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>6600</v>
       </c>
       <c r="C34" t="n">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
@@ -90618,14 +90608,14 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>comprehensive eye exam</t>
+          <t>eye operation cataract</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>6600</v>
       </c>
       <c r="C35" t="n">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
@@ -90641,14 +90631,14 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cost of cataract surgery</t>
+          <t>eyesight test</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>6600</v>
       </c>
       <c r="C36" t="n">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
@@ -90664,14 +90654,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>eye operation cataract</t>
+          <t>icl surgery</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>6600</v>
       </c>
       <c r="C37" t="n">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
@@ -90687,14 +90677,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>eyesight test</t>
+          <t>normal eye pressure</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>6600</v>
       </c>
       <c r="C38" t="n">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
@@ -90710,14 +90700,14 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>icl surgery</t>
+          <t>prk vs lasik</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>6600</v>
       </c>
       <c r="C39" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D39" s="12" t="inlineStr">
         <is>
@@ -90733,14 +90723,14 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>normal eye pressure</t>
+          <t>eye faults</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>6600</v>
       </c>
       <c r="C40" t="n">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
@@ -90756,14 +90746,14 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>prk vs lasik</t>
+          <t>ocular hypertension</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>6600</v>
+        <v>5400</v>
       </c>
       <c r="C41" t="n">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>

</xml_diff>